<commit_message>
updating json to excel and v1.0.0 template
</commit_message>
<xml_diff>
--- a/template/v1.0.0/vcds_template_1_0_0.xlsx
+++ b/template/v1.0.0/vcds_template_1_0_0.xlsx
@@ -370,7 +370,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1">
@@ -398,7 +398,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>A unique identifier for each combination of virus-host-sample within a study. The identifier is composed of a prefix, pmid, and a seven digit identifier.</t>
+          <t>A unique identifier for each combination of virus-host-sample within a study. The identifier is composed of a prefix, pmid, and a seven digit identifier. See http://purl.org/dc/elements/1.1/identifier</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -410,670 +410,670 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>study</t>
+          <t>group_id</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>An abbreviated citation for the study in the format Last name of first author, et al. Year Journal</t>
+          <t>An identifier for linking different sample types that originate from the same experimental conditions. The identifier is composed of letters and underscores (snakecase). Each identifier must be unique within the study. See http://purl.obolibrary.org/obo/NCIT_C82529</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Murrieta et al. 2021 PLoS Pathogens</t>
+          <t>a, group_A, aedes_Aegypti_Zika_virus</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>pmid</t>
+          <t>study</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>A unique integer used to identify works within the PubMed system. Not to be confused with a PubMed Central Identifier. See https://pmc.ncbi.nlm.nih.gov/about/public-access-info/ for additional details. See http://purl.obolibrary.org/obo/OBI_0001617 for definition.</t>
+          <t>An abbreviated citation for the study in the format Last name of first author, et al. Year Journal. See http://schema.org/citation</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>12345678</t>
+          <t>Murrieta et al. 2021 PLoS Pathogens</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>doi</t>
+          <t>pmid</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>A centrally registered identifier symbol used to uniquely identify objects given by International DOI Foundation. The DOI system is commonly used for electronic documents such as journal articles. See http://purl.obolibrary.org/obo/OBI_0002110.</t>
+          <t>A unique integer used to identify works within the PubMed system. Not to be confused with a PubMed Central Identifier. Review https://pmc.ncbi.nlm.nih.gov/about/public-access-info/ for additional details. See http://purl.obolibrary.org/obo/OBI_0001617</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>10.1603/ME10007</t>
+          <t>12345678</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>vector</t>
+          <t>doi</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>The Linnaean classification of the vector on which the experiment was performed, reported as a species binomial. See http://rs.tdwg.org/dwc/terms/scientificName</t>
+          <t>A centrally registered identifier symbol used to uniquely identify objects given by International DOI Foundation. The DOI system is commonly used for electronic documents such as journal articles. See http://purl.obolibrary.org/obo/OBI_0002110.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Aedes aegypti</t>
+          <t>10.1603/ME10007</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>vector_subspecies</t>
+          <t>vector</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vector subspecies.  A taxonomic category below that of species. See http://purl.obolibrary.org/obo/NCIT_C62700. </t>
+          <t>The Linnaean classification of the vector on which the experiment was performed, reported as a species binomial. See http://rs.tdwg.org/dwc/terms/scientificName</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Wiedemann</t>
+          <t>Aedes aegypti</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>vector_strain</t>
+          <t>vector_subspecies</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vector strain. A genetic variant within a species. See https://w3id.org/evorao/strain. </t>
+          <t>Vector subspecies. A taxonomic category below that of species. See http://purl.obolibrary.org/obo/NCIT_C62700</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>163/11, Zafferana</t>
+          <t>Wiedemann</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>vector_origin_country</t>
+          <t>vector_strain</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>The country that is the wild source for original vector collection. See http://rs.tdwg.org/dwc/terms/country</t>
+          <t>Vector strain. A genetic variant within a species. See https://w3id.org/evorao/strain</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>United States, Belgium, Central African Republic</t>
+          <t>163/11, Zafferana</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>vector_origin_locality</t>
+          <t>vector_origin_country</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>The location that is the wild source for original vector collection. See http://rs.tdwg.org/dwc/terms/locality</t>
+          <t>The country that is the wild source for original vector collection. See http://rs.tdwg.org/dwc/terms/country</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Pariquera-Açu Township, S.Paulo State, Kern County, California</t>
+          <t>United States, Belgium, Central African Republic</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>vector_origin_year</t>
+          <t>vector_origin_locality</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>The year when the wild source for original vector collection occurred. May also include season or other date information. Must contain a four digit year. See http://rs.tdwg.org/dwc/terms/year</t>
+          <t>The location that is the wild source for original vector collection. See http://rs.tdwg.org/dwc/terms/locality</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1995, Winter 2026</t>
+          <t>Pariquera-Açu Township, S.Paulo State, Kern County, California</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>vector_generation</t>
+          <t>vector_origin_year</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Vector generation in lab colony. See http://purl.obolibrary.org/obo/PCO_0000054</t>
+          <t>The year when the wild source for original vector collection occurred. May also include season or other date information. Must contain a four digit year. See http://rs.tdwg.org/dwc/terms/year</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>F2, F9-F10, 0</t>
+          <t>1995, Winter 2026</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>virus</t>
+          <t>vector_generation</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>The Linnaean classification of the virus with which the experiment was performed, reported as a species binomial. See http://rs.tdwg.org/dwc/terms/scientificName</t>
+          <t>Vector generation in lab colony. See http://purl.obolibrary.org/obo/PCO_0000054</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Yellow fever virus, Zika Virus, Orthoflavivirus zikaense</t>
+          <t>F2, F9-F10, 0</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>viral_lineage</t>
+          <t>virus</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Information about the genetic distinctness of the sequenced organism below the subspecies level, e.g., serovar, serotype, biotype, ecotype, or any relevant genetic typing schemes. See https://w3id.org/mixs/0000020</t>
+          <t>The Linnaean classification of the virus with which the experiment was performed, reported as a species binomial. See http://rs.tdwg.org/dwc/terms/scientificName</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>West African genotype, 2, Lineage 1</t>
+          <t>Yellow fever virus, Zika Virus, Orthoflavivirus zikaense</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>viral_strain</t>
+          <t>viral_lineage</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Identifier given to a genetic variant within a single species. See https://w3id.org/evorao/strain</t>
+          <t>Information about the genetic distinctness of the sequenced organism below the subspecies level, e.g., serovar, serotype, biotype, ecotype, or any relevant genetic typing schemes. See https://w3id.org/mixs/0000020</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>HJV 64A-1519, HJV B230, MMP1047</t>
+          <t>West African genotype, 2, Lineage 1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>viral_genbank_accession</t>
+          <t>viral_strain</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Accession number of an entry from the GenBank sequence database. See http://edamontology.org/data_2292</t>
+          <t>Identifier given to a genetic variant within a single species. See https://w3id.org/evorao/strain</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>KJ451624.1, U91870</t>
+          <t>HJV 64A-1519, HJV B230, MMP1047</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>recombinant_virus</t>
+          <t>viral_genbank_accession</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Is the virus derived from recombinant nucleic acid?</t>
+          <t>Accession number of an entry from the GenBank sequence database. See http://edamontology.org/data_2292</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>yes, no</t>
+          <t>KJ451624.1, U91870</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>wildtype_mutant</t>
+          <t>recombinant_virus</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Is the virus unmodified (wildtype) or has the genetic sequence of the virus been intentionally altered (mutant)? http://purl.obolibrary.org/obo/GENO_0000480</t>
+          <t>Is the virus derived from recombinant nucleic acid? See http://purl.bioontology.org/ontology/CSP/4005-0050</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>wildtype, mutant</t>
+          <t>yes, no</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>viral_origin_locality</t>
+          <t>wildtype_mutant</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>The location that is the wild source for original virus collection. See http://rs.tdwg.org/dwc/terms/locality</t>
+          <t>Is the virus unmodified (wildtype) or has the genetic sequence of the virus been intentionally altered (mutant)? http://purl.obolibrary.org/obo/GENO_0000480</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Zulia state, Venezuela, Zika Forest, Uganda</t>
+          <t>wildtype, mutant</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>viral_origin_year</t>
+          <t>viral_origin_locality</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>The year when the wild source for original virus collection occurred. May also include season or other date information. Must contain a four digit year. See http://rs.tdwg.org/dwc/terms/year</t>
+          <t>The location that is the wild source for original virus collection. See http://rs.tdwg.org/dwc/terms/locality</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1995, Winter 2026</t>
+          <t>Zulia state, Venezuela, Zika Forest, Uganda</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>viral_history_passage</t>
+          <t>viral_origin_year</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Cell type and passage number. See https://w3id.org/evorao/passage</t>
+          <t>The year when the wild source for original virus collection occurred. May also include season or other date information. Must contain a four digit year. See http://rs.tdwg.org/dwc/terms/year</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Vero, 2 passages, C6/36 3, Ae. triseriatus and Vero 12 alternate passages</t>
+          <t>1995, Winter 2026</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>viral_history_freshness</t>
+          <t>viral_history_passage</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Specifies the conditions under which the product was stored to maintain stability and integrity, such as temperature, buffer, and other environmental factors. See https://w3id.org/evorao/storageConditions</t>
+          <t>Cell type and passage number. See https://w3id.org/evorao/passage</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>fresh, frozen, -80ºC</t>
+          <t>Vero, 2 passages, C6/36 3, Ae. triseriatus and Vero 12 alternate passages</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>exposure_route</t>
+          <t>viral_history_freshness</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>How were vectors exposed. See http://purl.obolibrary.org/obo/ExO_0000055</t>
+          <t>Specifies the conditions under which the product was stored to maintain stability and integrity, such as temperature, buffer, and other environmental factors. See https://w3id.org/evorao/storageConditions</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>bloodmeal, intrathoracic injection, live animal</t>
+          <t>fresh, frozen, -80ºC</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>host_exposure</t>
+          <t>exposure_route</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Host species used for live animal exposure. See https://w3id.org/mixs/0001298</t>
+          <t xml:space="preserve"> The way a vector was exposed to a virus. See http://purl.obolibrary.org/obo/ExO_0000055</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Syrian hamster, chicken, American alligator</t>
+          <t>bloodmeal, intrathoracic injection, live animal</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>host_lineage_origin</t>
+          <t>host_exposure</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Host intraspecific lineage name, or origin. See https://w3id.org/mixs/0000020</t>
+          <t>Host species used for live animal exposure. See https://w3id.org/mixs/0001298</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mesocricetus auratus, C57BL/6</t>
+          <t>Syrian hamster, chicken, American alligator</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>diagnostic_viremia</t>
+          <t>host_lineage_origin</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Diagnostic method used, if any, for measuring host viremia. See http://id.nlm.nih.gov/mesh/D019411</t>
+          <t>Host intraspecific lineage name, or origin. See https://w3id.org/mixs/0000020</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>plaque assay, qRT-PCR</t>
+          <t>Mesocricetus auratus, C57BL/6</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>titer</t>
+          <t>diagnostic_viremia</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Concentration of virus in bloodmeal, intrathoracic inoculation or host viremia if live animal. See http://purl.obolibrary.org/obo/VO_0000555</t>
+          <t>Diagnostic method used, if any, for measuring host viremia. See http://id.nlm.nih.gov/mesh/D019411</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>&gt;8.8, 44000000, 1E7.1</t>
+          <t>plaque assay, qRT-PCR</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>titer_units</t>
+          <t>titer</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Unit of measure for titer concentration. See http://purl.obolibrary.org/obo/NCIT_C67375</t>
+          <t>Concentration of virus in bloodmeal, intrathoracic inoculation or host viremia if live animal. See http://purl.obolibrary.org/obo/VO_0000555</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>log10 FFU/ml, viral RNA/ml, MID50/ml</t>
+          <t>&gt;8.8, 44000000, 1E7.1</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>dose</t>
+          <t>titer_units</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Dose of live virus injected via intrathoracic inoculation, if applicable. See http://purl.obolibrary.org/obo/NCIT_C25488</t>
+          <t>Unit of measure for titer concentration. See http://purl.obolibrary.org/obo/NCIT_C67375</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>&lt;0.5, 3.2</t>
+          <t>log10 FFU/ml, viral RNA/ml, MID50/ml</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>dose_units</t>
+          <t>dose</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Unit of measure for the dose. See http://purl.obolibrary.org/obo/NCIT_C48463</t>
+          <t>Dose of live virus injected via intrathoracic inoculation, if applicable. See http://purl.obolibrary.org/obo/NCIT_C25488</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>TCID50, PFU, log10 TCID50, log10 PFU</t>
+          <t>&lt;0.5, 3.2</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>mean_temp_reared</t>
+          <t>dose_units</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Average temperature recorded during rearing in celsius. See http://www.ebi.ac.uk/efo/EFO_0001702</t>
+          <t>Unit of measure for the dose. See http://purl.obolibrary.org/obo/NCIT_C48463</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>25.2, 30, 18, 27.6</t>
+          <t>TCID50, PFU, log10 TCID50, log10 PFU</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ampliture_temp_reared</t>
+          <t>mean_temp_reared</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Ampliture of temperature at which vectors are reared in Celsius. See http://biomodels.net/SBO/SBO_0000492</t>
+          <t>Average temperature during rearing in Celsius. See http://www.ebi.ac.uk/efo/EFO_0001702</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>5, 3, 2</t>
+          <t>25.2, 30, 18, 27.6</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>relative_humidity_reared</t>
+          <t>amplitude_temp_reared</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Percent relative humidity at which vectors are reared in Celsius. See http://purl.allotrope.org/ontologies/result#AFR_0002614</t>
+          <t>Amplitude of temperature at which vectors are reared in Celsius. See http://purl.obolibrary.org/obo/NCIT_C70831</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>99, 50-60, 2</t>
+          <t>5, 3, 2</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>mean_temp_eit</t>
+          <t>relative_humidity_reared</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Average temperature at which extrinsic incubation happens in Celsius. See http://www.ebi.ac.uk/efo/EFO_0001702</t>
+          <t>Percent relative humidity at which vectors are reared. See http://purl.allotrope.org/ontologies/result#AFR_0002614</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>25.2, 30, 18, 27.6</t>
+          <t>99, 50-60, 2</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ampliture_temp_eit</t>
+          <t>mean_temp_eit</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Ampliture of temperature at which extrinsic incubation happens in Celsius. See http://biomodels.net/SBO/SBO_0000492</t>
+          <t>Average temperature at which extrinsic incubation happens in Celsius. See http://www.ebi.ac.uk/efo/EFO_0001702</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>5, 3, 2</t>
+          <t>25.2, 30, 18, 27.6</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>relative_humidity_eit</t>
+          <t>amplitude_temp_eit</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Percent relative humidity at which vectors are reared in Celsius. See http://purl.allotrope.org/ontologies/result#AFR_0002614</t>
+          <t>Amplitude of temperature at which extrinsic incubation happens in Celsius. See http://purl.obolibrary.org/obo/NCIT_C70831</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>99, 50-60, 2</t>
+          <t>5, 3, 2</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>dpi</t>
+          <t>relative_humidity_eit</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Days post-infection. See http://purl.obolibrary.org/obo/UO_0000003</t>
+          <t>Percent relative humidity at which vectors are reared. See http://purl.allotrope.org/ontologies/result#AFR_0002614</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>5, 3-10, &gt;2</t>
+          <t>99, 50-60, 2</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>coinfected</t>
+          <t>dpi</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Is your mosquito knowingly infected with another organism. See http://www.ebi.ac.uk/efo/EFO_0010716</t>
+          <t>Days post-infection. See http://purl.obolibrary.org/obo/UO_0000003</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>yes, no</t>
+          <t>5, 3-10, &gt;2</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>coinfected</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Vector sample part used to establish infection. See http://purl.obolibrary.org/obo/OBI_0100051</t>
+          <t>Is your mosquito knowingly infected with another organism? See http://www.ebi.ac.uk/efo/EFO_0010716</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>body, head, salivary glands</t>
+          <t>yes, no</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>diagnostic</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>How vector infection was established. See http://id.nlm.nih.gov/mesh/D019411</t>
+          <t>Vector sample part used to establish infection. See http://purl.obolibrary.org/obo/OBI_0100051</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>qRT-PCR, IFA, plaque assay</t>
+          <t>body, head, salivary glands</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>tested</t>
+          <t>diagnostic</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Number of vectors tested for infection. See http://purl.obolibrary.org/obo/NCIT_C25463</t>
+          <t>How vector infection was established. See http://id.nlm.nih.gov/mesh/D019411</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>1, 1000, 42</t>
+          <t>qRT-PCR, IFA, plaque assay</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>tested</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1090,100 +1090,117 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>transmission_recipient</t>
+          <t>positive</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Host species used for live animal exposure.</t>
+          <t>Number of vectors tested for infection. See http://purl.obolibrary.org/obo/NCIT_C25463</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>suckling mouse, chicken</t>
+          <t>1, 1000, 42</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>transmission_diagnostic</t>
+          <t>transmission_recipient</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Diagnostic method used to detect infection in animal. See http://id.nlm.nih.gov/mesh/D019411</t>
+          <t>Host species used for live animal exposure.</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>seroconversion, death, plaque assay</t>
+          <t>suckling mouse, chicken</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>num_vector_fed</t>
+          <t>transmission_diagnostic</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Number of vectors fed on the live animal. See http://purl.obolibrary.org/obo/NCIT_C25463</t>
+          <t>Diagnostic method used to detect infection in animal. See http://id.nlm.nih.gov/mesh/D019411</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>1, 1000, 42</t>
+          <t>seroconversion, death, plaque assay</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>num_vector_positive</t>
+          <t>num_vector_fed</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Number of infected vectors that fed on the live animal. See http://purl.obolibrary.org/obo/NCIT_C25463</t>
+          <t>Number of vectors fed on the live animal. See http://purl.obolibrary.org/obo/NCIT_C25463</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>1, 500, 21</t>
+          <t>1, 1000, 42</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>num_recipients_tested</t>
+          <t>num_vector_positive</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Number of recipient animals tested for infection. See http://purl.obolibrary.org/obo/NCIT_C25463</t>
+          <t>Number of infected vectors that fed on the live animal. See http://purl.obolibrary.org/obo/NCIT_C25463</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>10, 501, 121</t>
+          <t>1, 500, 21</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>num_recipients_tested</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Number of recipient animals tested for infection. See http://purl.obolibrary.org/obo/NCIT_C25463</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>10, 501, 121</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
           <t>num_recipients_positive</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>Number of recipient animals that tested positive. See http://purl.obolibrary.org/obo/NCIT_C25463</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>5, 52, 12</t>
         </is>
@@ -1198,7 +1215,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:AU2"/>
+  <dimension ref="A1:AV2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1">
@@ -1209,230 +1226,235 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>group_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>study</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>pmid</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>doi</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>vector</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>vector_subspecies</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>vector_strain</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>vector_origin_country</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>vector_origin_locality</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>vector_origin_year</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>vector_generation</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>virus</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>viral_lineage</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>viral_strain</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>viral_genbank_accession</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>recombinant_virus</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>wildtype_mutant</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>viral_origin_locality</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>viral_origin_year</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>viral_history_passage</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>viral_history_freshness</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>exposure_route</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>host_exposure</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>host_lineage_origin</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>diagnostic_viremia</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>titer</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>titer_units</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>dose</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>dose_units</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>mean_temp_reared</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>ampliture_temp_reared</t>
-        </is>
-      </c>
       <c r="AF1" t="inlineStr">
         <is>
+          <t>amplitude_temp_reared</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
           <t>relative_humidity_reared</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>mean_temp_eit</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
-        <is>
-          <t>ampliture_temp_eit</t>
-        </is>
-      </c>
       <c r="AI1" t="inlineStr">
         <is>
+          <t>amplitude_temp_eit</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
           <t>relative_humidity_eit</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>dpi</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>coinfected</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>sample</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>diagnostic</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>positive</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>transmission_recipient</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>transmission_diagnostic</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>num_vector_fed</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>num_vector_positive</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>num_recipients_tested</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>num_recipients_positive</t>
         </is>
@@ -1670,6 +1692,11 @@
         </is>
       </c>
       <c r="AU2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
         <is>
           <t/>
         </is>

</xml_diff>

<commit_message>
chore: regenerate excel templates
</commit_message>
<xml_diff>
--- a/template/v1.0.0/vcds_template_1_0_0.xlsx
+++ b/template/v1.0.0/vcds_template_1_0_0.xlsx
@@ -370,7 +370,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1">
@@ -398,682 +398,682 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>A unique identifier for each combination of virus-host-sample within a study. The identifier is composed of a prefix, pmid, and a seven digit identifier. See http://purl.org/dc/elements/1.1/identifier</t>
+          <t>This grouping identifier connects different sample types that originate from the same experimental conditions and virus-vector combination within a study. The identifier is composed of a prefix, pmid, and a seven digit identifier. See http://purl.org/dc/elements/1.1/identifier</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>cmt_12345678_0000001, aed_87654321_0000001, tck_1_0000001</t>
+          <t>cmt_12345678_0000001, aed_87654321_0000001, tck_1_0001111</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>group_id</t>
+          <t>study</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>An identifier for linking different sample types that originate from the same experimental conditions. The identifier is composed of letters and underscores (snakecase). Each identifier must be unique within the study. See http://purl.obolibrary.org/obo/NCIT_C82529</t>
+          <t>An abbreviated citation for the study in the format Last name of first author, et al. Year Journal. See http://schema.org/citation</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>a, group_A, aedes_Aegypti_Zika_virus</t>
+          <t>Murrieta et al. 2021 PLoS Pathogens</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>study</t>
+          <t>pmid</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>An abbreviated citation for the study in the format Last name of first author, et al. Year Journal. See http://schema.org/citation</t>
+          <t>A unique integer used to identify works within the PubMed system. Not to be confused with a PubMed Central Identifier. Review https://pmc.ncbi.nlm.nih.gov/about/public-access-info/ for additional details. See http://purl.obolibrary.org/obo/OBI_0001617</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Murrieta et al. 2021 PLoS Pathogens</t>
+          <t>12345678</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>pmid</t>
+          <t>doi</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>A unique integer used to identify works within the PubMed system. Not to be confused with a PubMed Central Identifier. Review https://pmc.ncbi.nlm.nih.gov/about/public-access-info/ for additional details. See http://purl.obolibrary.org/obo/OBI_0001617</t>
+          <t>A centrally registered identifier symbol used to uniquely identify objects given by International DOI Foundation. The DOI system is commonly used for electronic documents such as journal articles. See http://purl.obolibrary.org/obo/OBI_0002110.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>12345678</t>
+          <t>10.1603/ME10007</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>doi</t>
+          <t>vector</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>A centrally registered identifier symbol used to uniquely identify objects given by International DOI Foundation. The DOI system is commonly used for electronic documents such as journal articles. See http://purl.obolibrary.org/obo/OBI_0002110.</t>
+          <t>The Linnaean classification of the vector on which the experiment was performed, reported as a species binomial. See http://rs.tdwg.org/dwc/terms/scientificName</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>10.1603/ME10007</t>
+          <t>Aedes aegypti</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>vector</t>
+          <t>vector_subspecies</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>The Linnaean classification of the vector on which the experiment was performed, reported as a species binomial. See http://rs.tdwg.org/dwc/terms/scientificName</t>
+          <t>Vector subspecies. A taxonomic category below that of species. See http://purl.obolibrary.org/obo/NCIT_C62700</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Aedes aegypti</t>
+          <t>Wiedemann</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>vector_subspecies</t>
+          <t>vector_strain</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Vector subspecies. A taxonomic category below that of species. See http://purl.obolibrary.org/obo/NCIT_C62700</t>
+          <t>Vector strain. A genetic variant within a species. See https://w3id.org/evorao/strain</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Wiedemann</t>
+          <t>163/11, Zafferana</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>vector_strain</t>
+          <t>vector_origin_country</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Vector strain. A genetic variant within a species. See https://w3id.org/evorao/strain</t>
+          <t>The country that is the wild source for original vector collection. See http://rs.tdwg.org/dwc/terms/country</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>163/11, Zafferana</t>
+          <t>United States, Belgium, Central African Republic</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>vector_origin_country</t>
+          <t>vector_origin_locality</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>The country that is the wild source for original vector collection. See http://rs.tdwg.org/dwc/terms/country</t>
+          <t>The location that is the wild source for original vector collection. See http://rs.tdwg.org/dwc/terms/locality</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>United States, Belgium, Central African Republic</t>
+          <t>Pariquera-Açu Township, S.Paulo State, Kern County, California</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>vector_origin_locality</t>
+          <t>vector_origin_year</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>The location that is the wild source for original vector collection. See http://rs.tdwg.org/dwc/terms/locality</t>
+          <t>The year when the wild source for original vector collection occurred. May also include season or other date information. Must contain a four digit year. See http://rs.tdwg.org/dwc/terms/year</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Pariquera-Açu Township, S.Paulo State, Kern County, California</t>
+          <t>1995, Winter 2026</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>vector_origin_year</t>
+          <t>vector_generation</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>The year when the wild source for original vector collection occurred. May also include season or other date information. Must contain a four digit year. See http://rs.tdwg.org/dwc/terms/year</t>
+          <t>Vector generation in lab colony. See http://purl.obolibrary.org/obo/PCO_0000054</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1995, Winter 2026</t>
+          <t>F2, F9-F10, 0</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>vector_generation</t>
+          <t>virus</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Vector generation in lab colony. See http://purl.obolibrary.org/obo/PCO_0000054</t>
+          <t>The Linnaean classification of the virus with which the experiment was performed, reported as a species binomial. See http://rs.tdwg.org/dwc/terms/scientificName</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>F2, F9-F10, 0</t>
+          <t>Yellow fever virus, Zika Virus, Orthoflavivirus zikaense</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>virus</t>
+          <t>viral_lineage</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>The Linnaean classification of the virus with which the experiment was performed, reported as a species binomial. See http://rs.tdwg.org/dwc/terms/scientificName</t>
+          <t>Information about the genetic distinctness of the sequenced organism below the subspecies level, e.g., serovar, serotype, biotype, ecotype, or any relevant genetic typing schemes. See https://w3id.org/mixs/0000020</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Yellow fever virus, Zika Virus, Orthoflavivirus zikaense</t>
+          <t>West African genotype, 2, Lineage 1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>viral_lineage</t>
+          <t>viral_strain</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Information about the genetic distinctness of the sequenced organism below the subspecies level, e.g., serovar, serotype, biotype, ecotype, or any relevant genetic typing schemes. See https://w3id.org/mixs/0000020</t>
+          <t>Identifier given to a genetic variant within a single species. See https://w3id.org/evorao/strain</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>West African genotype, 2, Lineage 1</t>
+          <t>HJV 64A-1519, HJV B230, MMP1047</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>viral_strain</t>
+          <t>viral_genbank_accession</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Identifier given to a genetic variant within a single species. See https://w3id.org/evorao/strain</t>
+          <t>Accession number of an entry from the GenBank sequence database. See http://edamontology.org/data_2292</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>HJV 64A-1519, HJV B230, MMP1047</t>
+          <t>KJ451624.1, U91870</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>viral_genbank_accession</t>
+          <t>recombinant_virus</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Accession number of an entry from the GenBank sequence database. See http://edamontology.org/data_2292</t>
+          <t>Is the virus derived from recombinant nucleic acid? See http://purl.bioontology.org/ontology/CSP/4005-0050</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>KJ451624.1, U91870</t>
+          <t>yes, no</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>recombinant_virus</t>
+          <t>wildtype_mutant</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Is the virus derived from recombinant nucleic acid? See http://purl.bioontology.org/ontology/CSP/4005-0050</t>
+          <t>Is the virus unmodified (wildtype) or has the genetic sequence of the virus been intentionally altered (mutant)? http://purl.obolibrary.org/obo/GENO_0000480</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>yes, no</t>
+          <t>wildtype, mutant</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>wildtype_mutant</t>
+          <t>viral_origin_locality</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Is the virus unmodified (wildtype) or has the genetic sequence of the virus been intentionally altered (mutant)? http://purl.obolibrary.org/obo/GENO_0000480</t>
+          <t>The location that is the wild source for original virus collection. See http://rs.tdwg.org/dwc/terms/locality</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>wildtype, mutant</t>
+          <t>Zulia state, Venezuela, Zika Forest, Uganda</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>viral_origin_locality</t>
+          <t>viral_origin_year</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>The location that is the wild source for original virus collection. See http://rs.tdwg.org/dwc/terms/locality</t>
+          <t>The year when the wild source for original virus collection occurred. May also include season or other date information. Must contain a four digit year. See http://rs.tdwg.org/dwc/terms/year</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Zulia state, Venezuela, Zika Forest, Uganda</t>
+          <t>1995, Winter 2026</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>viral_origin_year</t>
+          <t>viral_history_passage</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>The year when the wild source for original virus collection occurred. May also include season or other date information. Must contain a four digit year. See http://rs.tdwg.org/dwc/terms/year</t>
+          <t>Cell type and passage number. See https://w3id.org/evorao/passage</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1995, Winter 2026</t>
+          <t>Vero, 2 passages, C6/36 3, Ae. triseriatus and Vero 12 alternate passages</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>viral_history_passage</t>
+          <t>viral_history_freshness</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Cell type and passage number. See https://w3id.org/evorao/passage</t>
+          <t>Specifies the conditions under which the product was stored to maintain stability and integrity, such as temperature, buffer, and other environmental factors. See https://w3id.org/evorao/storageConditions</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Vero, 2 passages, C6/36 3, Ae. triseriatus and Vero 12 alternate passages</t>
+          <t>fresh, frozen, -80ºC</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>viral_history_freshness</t>
+          <t>exposure_route</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Specifies the conditions under which the product was stored to maintain stability and integrity, such as temperature, buffer, and other environmental factors. See https://w3id.org/evorao/storageConditions</t>
+          <t xml:space="preserve"> The way a vector was exposed to a virus. See http://purl.obolibrary.org/obo/ExO_0000055</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>fresh, frozen, -80ºC</t>
+          <t>bloodmeal, intrathoracic injection, live animal</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>exposure_route</t>
+          <t>host_exposure</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> The way a vector was exposed to a virus. See http://purl.obolibrary.org/obo/ExO_0000055</t>
+          <t>Host species used for live animal exposure. See https://w3id.org/mixs/0001298</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>bloodmeal, intrathoracic injection, live animal</t>
+          <t>Syrian hamster, chicken, American alligator</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>host_exposure</t>
+          <t>host_lineage_origin</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Host species used for live animal exposure. See https://w3id.org/mixs/0001298</t>
+          <t>Host intraspecific lineage name, or origin. See https://w3id.org/mixs/0000020</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Syrian hamster, chicken, American alligator</t>
+          <t>Mesocricetus auratus, C57BL/6</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>host_lineage_origin</t>
+          <t>diagnostic_viremia</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Host intraspecific lineage name, or origin. See https://w3id.org/mixs/0000020</t>
+          <t>Diagnostic method used, if any, for measuring host viremia. See http://id.nlm.nih.gov/mesh/D019411</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mesocricetus auratus, C57BL/6</t>
+          <t>plaque assay, qRT-PCR</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>diagnostic_viremia</t>
+          <t>titer</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Diagnostic method used, if any, for measuring host viremia. See http://id.nlm.nih.gov/mesh/D019411</t>
+          <t>Concentration of virus in bloodmeal, intrathoracic inoculation or host viremia if live animal. See http://purl.obolibrary.org/obo/VO_0000555</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>plaque assay, qRT-PCR</t>
+          <t>&gt;8.8, 44000000, 1E7.1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>titer</t>
+          <t>titer_units</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Concentration of virus in bloodmeal, intrathoracic inoculation or host viremia if live animal. See http://purl.obolibrary.org/obo/VO_0000555</t>
+          <t>Unit of measure for titer concentration. See http://purl.obolibrary.org/obo/NCIT_C67375</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>&gt;8.8, 44000000, 1E7.1</t>
+          <t>log10 FFU/ml, viral RNA/ml, MID50/ml</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>titer_units</t>
+          <t>dose</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Unit of measure for titer concentration. See http://purl.obolibrary.org/obo/NCIT_C67375</t>
+          <t>Dose of live virus injected via intrathoracic inoculation, if applicable. See http://purl.obolibrary.org/obo/NCIT_C25488</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>log10 FFU/ml, viral RNA/ml, MID50/ml</t>
+          <t>&lt;0.5, 3.2</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>dose</t>
+          <t>dose_units</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Dose of live virus injected via intrathoracic inoculation, if applicable. See http://purl.obolibrary.org/obo/NCIT_C25488</t>
+          <t>Unit of measure for the dose. See http://purl.obolibrary.org/obo/NCIT_C48463</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>&lt;0.5, 3.2</t>
+          <t>TCID50, PFU, log10 TCID50, log10 PFU</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>dose_units</t>
+          <t>mean_temp_reared</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Unit of measure for the dose. See http://purl.obolibrary.org/obo/NCIT_C48463</t>
+          <t>Average temperature during rearing in Celsius. See http://www.ebi.ac.uk/efo/EFO_0001702</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>TCID50, PFU, log10 TCID50, log10 PFU</t>
+          <t>25.2, 30, 18, 27.6</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>mean_temp_reared</t>
+          <t>amplitude_temp_reared</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Average temperature during rearing in Celsius. See http://www.ebi.ac.uk/efo/EFO_0001702</t>
+          <t>Amplitude of temperature at which vectors are reared in Celsius. See http://purl.obolibrary.org/obo/NCIT_C70831</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>25.2, 30, 18, 27.6</t>
+          <t>5, 3, 2</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>amplitude_temp_reared</t>
+          <t>relative_humidity_reared</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Amplitude of temperature at which vectors are reared in Celsius. See http://purl.obolibrary.org/obo/NCIT_C70831</t>
+          <t>Percent relative humidity at which vectors are reared. See http://purl.allotrope.org/ontologies/result#AFR_0002614</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>5, 3, 2</t>
+          <t>99, 50-60, 2</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>relative_humidity_reared</t>
+          <t>mean_temp_eit</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Percent relative humidity at which vectors are reared. See http://purl.allotrope.org/ontologies/result#AFR_0002614</t>
+          <t>Average temperature at which extrinsic incubation happens in Celsius. See http://www.ebi.ac.uk/efo/EFO_0001702</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>99, 50-60, 2</t>
+          <t>25.2, 30, 18, 27.6</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>mean_temp_eit</t>
+          <t>amplitude_temp_eit</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Average temperature at which extrinsic incubation happens in Celsius. See http://www.ebi.ac.uk/efo/EFO_0001702</t>
+          <t>Amplitude of temperature at which extrinsic incubation happens in Celsius. See http://purl.obolibrary.org/obo/NCIT_C70831</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>25.2, 30, 18, 27.6</t>
+          <t>5, 3, 2</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>amplitude_temp_eit</t>
+          <t>relative_humidity_eit</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Amplitude of temperature at which extrinsic incubation happens in Celsius. See http://purl.obolibrary.org/obo/NCIT_C70831</t>
+          <t>Percent relative humidity at which vectors are reared. See http://purl.allotrope.org/ontologies/result#AFR_0002614</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>5, 3, 2</t>
+          <t>99, 50-60, 2</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>relative_humidity_eit</t>
+          <t>dpi</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Percent relative humidity at which vectors are reared. See http://purl.allotrope.org/ontologies/result#AFR_0002614</t>
+          <t>Days post-infection. See http://purl.obolibrary.org/obo/UO_0000003</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>99, 50-60, 2</t>
+          <t>5, 3-10, &gt;2</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>dpi</t>
+          <t>coinfected</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Days post-infection. See http://purl.obolibrary.org/obo/UO_0000003</t>
+          <t>Is your mosquito knowingly infected with another organism? See http://www.ebi.ac.uk/efo/EFO_0010716</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>5, 3-10, &gt;2</t>
+          <t>yes, no</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>coinfected</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Is your mosquito knowingly infected with another organism? See http://www.ebi.ac.uk/efo/EFO_0010716</t>
+          <t>Vector sample part used to establish infection. See http://purl.obolibrary.org/obo/OBI_0100051</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>yes, no</t>
+          <t>body, head, salivary glands</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>diagnostic</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Vector sample part used to establish infection. See http://purl.obolibrary.org/obo/OBI_0100051</t>
+          <t>How vector infection was established. See http://id.nlm.nih.gov/mesh/D019411</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>body, head, salivary glands</t>
+          <t>qRT-PCR, IFA, plaque assay</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>diagnostic</t>
+          <t>tested</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>How vector infection was established. See http://id.nlm.nih.gov/mesh/D019411</t>
+          <t>Number of vectors tested for infection. See http://purl.obolibrary.org/obo/NCIT_C25463</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>qRT-PCR, IFA, plaque assay</t>
+          <t>1, 1000, 42</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>tested</t>
+          <t>positive</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1090,117 +1090,100 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>transmission_recipient</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Number of vectors tested for infection. See http://purl.obolibrary.org/obo/NCIT_C25463</t>
+          <t>Host species used for live animal exposure.</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>1, 1000, 42</t>
+          <t>suckling mouse, chicken</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>transmission_recipient</t>
+          <t>transmission_diagnostic</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Host species used for live animal exposure.</t>
+          <t>Diagnostic method used to detect infection in animal. See http://id.nlm.nih.gov/mesh/D019411</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>suckling mouse, chicken</t>
+          <t>seroconversion, death, plaque assay</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>transmission_diagnostic</t>
+          <t>num_vector_fed</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Diagnostic method used to detect infection in animal. See http://id.nlm.nih.gov/mesh/D019411</t>
+          <t>Number of vectors fed on the live animal. See http://purl.obolibrary.org/obo/NCIT_C25463</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>seroconversion, death, plaque assay</t>
+          <t>1, 1000, 42</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>num_vector_fed</t>
+          <t>num_vector_positive</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Number of vectors fed on the live animal. See http://purl.obolibrary.org/obo/NCIT_C25463</t>
+          <t>Number of infected vectors that fed on the live animal. See http://purl.obolibrary.org/obo/NCIT_C25463</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>1, 1000, 42</t>
+          <t>1, 500, 21</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>num_vector_positive</t>
+          <t>num_recipients_tested</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Number of infected vectors that fed on the live animal. See http://purl.obolibrary.org/obo/NCIT_C25463</t>
+          <t>Number of recipient animals tested for infection. See http://purl.obolibrary.org/obo/NCIT_C25463</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>1, 500, 21</t>
+          <t>10, 501, 121</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>num_recipients_tested</t>
+          <t>num_recipients_positive</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Number of recipient animals tested for infection. See http://purl.obolibrary.org/obo/NCIT_C25463</t>
+          <t>Number of recipient animals that tested positive. See http://purl.obolibrary.org/obo/NCIT_C25463</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
-        <is>
-          <t>10, 501, 121</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>num_recipients_positive</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Number of recipient animals that tested positive. See http://purl.obolibrary.org/obo/NCIT_C25463</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
         <is>
           <t>5, 52, 12</t>
         </is>
@@ -1215,7 +1198,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:AV2"/>
+  <dimension ref="A1:AU2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1">
@@ -1226,235 +1209,230 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>group_id</t>
+          <t>study</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>study</t>
+          <t>pmid</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>pmid</t>
+          <t>doi</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>doi</t>
+          <t>vector</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>vector</t>
+          <t>vector_subspecies</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>vector_subspecies</t>
+          <t>vector_strain</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>vector_strain</t>
+          <t>vector_origin_country</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>vector_origin_country</t>
+          <t>vector_origin_locality</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>vector_origin_locality</t>
+          <t>vector_origin_year</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>vector_origin_year</t>
+          <t>vector_generation</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>vector_generation</t>
+          <t>virus</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>virus</t>
+          <t>viral_lineage</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>viral_lineage</t>
+          <t>viral_strain</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>viral_strain</t>
+          <t>viral_genbank_accession</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>viral_genbank_accession</t>
+          <t>recombinant_virus</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>recombinant_virus</t>
+          <t>wildtype_mutant</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>wildtype_mutant</t>
+          <t>viral_origin_locality</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>viral_origin_locality</t>
+          <t>viral_origin_year</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>viral_origin_year</t>
+          <t>viral_history_passage</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>viral_history_passage</t>
+          <t>viral_history_freshness</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>viral_history_freshness</t>
+          <t>exposure_route</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>exposure_route</t>
+          <t>host_exposure</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>host_exposure</t>
+          <t>host_lineage_origin</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
         <is>
-          <t>host_lineage_origin</t>
+          <t>diagnostic_viremia</t>
         </is>
       </c>
       <c r="Z1" t="inlineStr">
         <is>
-          <t>diagnostic_viremia</t>
+          <t>titer</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr">
         <is>
-          <t>titer</t>
+          <t>titer_units</t>
         </is>
       </c>
       <c r="AB1" t="inlineStr">
         <is>
-          <t>titer_units</t>
+          <t>dose</t>
         </is>
       </c>
       <c r="AC1" t="inlineStr">
         <is>
-          <t>dose</t>
+          <t>dose_units</t>
         </is>
       </c>
       <c r="AD1" t="inlineStr">
         <is>
-          <t>dose_units</t>
+          <t>mean_temp_reared</t>
         </is>
       </c>
       <c r="AE1" t="inlineStr">
         <is>
-          <t>mean_temp_reared</t>
+          <t>amplitude_temp_reared</t>
         </is>
       </c>
       <c r="AF1" t="inlineStr">
         <is>
-          <t>amplitude_temp_reared</t>
+          <t>relative_humidity_reared</t>
         </is>
       </c>
       <c r="AG1" t="inlineStr">
         <is>
-          <t>relative_humidity_reared</t>
+          <t>mean_temp_eit</t>
         </is>
       </c>
       <c r="AH1" t="inlineStr">
         <is>
-          <t>mean_temp_eit</t>
+          <t>amplitude_temp_eit</t>
         </is>
       </c>
       <c r="AI1" t="inlineStr">
         <is>
-          <t>amplitude_temp_eit</t>
+          <t>relative_humidity_eit</t>
         </is>
       </c>
       <c r="AJ1" t="inlineStr">
         <is>
-          <t>relative_humidity_eit</t>
+          <t>dpi</t>
         </is>
       </c>
       <c r="AK1" t="inlineStr">
         <is>
-          <t>dpi</t>
+          <t>coinfected</t>
         </is>
       </c>
       <c r="AL1" t="inlineStr">
         <is>
-          <t>coinfected</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="AM1" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>diagnostic</t>
         </is>
       </c>
       <c r="AN1" t="inlineStr">
         <is>
-          <t>diagnostic</t>
+          <t>tested</t>
         </is>
       </c>
       <c r="AO1" t="inlineStr">
         <is>
-          <t>tested</t>
+          <t>positive</t>
         </is>
       </c>
       <c r="AP1" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>transmission_recipient</t>
         </is>
       </c>
       <c r="AQ1" t="inlineStr">
         <is>
-          <t>transmission_recipient</t>
+          <t>transmission_diagnostic</t>
         </is>
       </c>
       <c r="AR1" t="inlineStr">
         <is>
-          <t>transmission_diagnostic</t>
+          <t>num_vector_fed</t>
         </is>
       </c>
       <c r="AS1" t="inlineStr">
         <is>
-          <t>num_vector_fed</t>
+          <t>num_vector_positive</t>
         </is>
       </c>
       <c r="AT1" t="inlineStr">
         <is>
-          <t>num_vector_positive</t>
+          <t>num_recipients_tested</t>
         </is>
       </c>
       <c r="AU1" t="inlineStr">
-        <is>
-          <t>num_recipients_tested</t>
-        </is>
-      </c>
-      <c r="AV1" t="inlineStr">
         <is>
           <t>num_recipients_positive</t>
         </is>
@@ -1692,11 +1670,6 @@
         </is>
       </c>
       <c r="AU2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AV2" t="inlineStr">
         <is>
           <t/>
         </is>

</xml_diff>